<commit_message>
Jerarquías sin relleno de ceros, vista previa de planillas del historial, hora de Chile y planillas de Modelos actualizadas
- Modelos (Maquinarias, Vehículos/Camiones): las jerarquías de nivel 1 y 2 ya no se completan con ceros hasta 18 dígitos (salen de 5 y 10 dígitos, igual que el código del diccionario SAP).
- Historial: botón "Vista previa" en la página de cada material, que muestra en pantalla la planilla guardada antes de descargarla (solo las filas del material, o el inicio de toda la planilla).
- Fechas del historial en hora de Chile (America/Santiago) en vez de la hora del servidor (UTC); los registros ya guardados se corrigen una sola vez.
- Planilla de Maquinarias actualizada (nuevas categorías, rangos de las listas desplegables ajustados) y MAQ. AGRICOLA quitado de la planilla de Vehículos y Camiones.
- Ajustes de contador: +3 a ZVEH, ZMAQ y ZCAM (una sola vez).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/Unidades/plantilla_modelos_ZVEH_ZCAM.xlsx
+++ b/data/reference/Unidades/plantilla_modelos_ZVEH_ZCAM.xlsx
@@ -13396,7 +13396,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -13446,17 +13446,6 @@
       </c>
       <c r="C4" s="6" t="s">
         <v>551</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>552</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>